<commit_message>
Phase 2 EfficientNet-B0 results: fruits_quality, mendeley_fruits, lemon. Update README with changelog.
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -1073,17 +1073,32 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>KFS-R18-C2-FS
+F1:  98.1%
+ACC: 98.9%
+MCC: 0.988
+AUC: 0.9999
+Time: 3.1 min</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-R18-C3-FS
+F1:  96.1%
+ACC: 97.9%
+MCC: 0.977
+AUC: 0.9996
+Time: 62.9 min</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-R18-C4-FS
+F1:  97.9%
+ACC: 98.8%
+MCC: 0.987
+AUC: 0.9999
+Time: 60.1 min</t>
         </is>
       </c>
     </row>
@@ -2544,8 +2559,8 @@
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
@@ -2603,22 +2618,42 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB0-C1-ST
+F1:  84.7%
+ACC: 84.7%
+MCC: 0.695
+AUC: 0.9182
+Time: 21.1 min</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB0-C2-ST
+F1:  86.1%
+ACC: 86.1%
+MCC: 0.732
+AUC: 0.8889
+Time: 19.8 min</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB0-C3-ST
+F1:  81.9%
+ACC: 81.9%
+MCC: 0.641
+AUC: 0.9275
+Time: 19.7 min</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB0-C4-ST
+F1:  86.1%
+ACC: 86.1%
+MCC: 0.727
+AUC: 0.8827
+Time: 19.8 min</t>
         </is>
       </c>
     </row>
@@ -2673,22 +2708,42 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB0-C1-ST
+F1:  94.6%
+ACC: 94.6%
+MCC: 0.896
+AUC: 0.9924
+Time: 22.0 min</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB0-C2-ST
+F1:  91.5%
+ACC: 91.5%
+MCC: 0.843
+AUC: 0.9730
+Time: 22.0 min</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB0-C3-ST
+F1:  97.0%
+ACC: 97.0%
+MCC: 0.940
+AUC: 0.9963
+Time: 21.8 min</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB0-C4-ST
+F1:  95.8%
+ACC: 95.8%
+MCC: 0.917
+AUC: 0.9855
+Time: 21.8 min</t>
         </is>
       </c>
     </row>
@@ -2743,22 +2798,42 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB0-C1-ST
+F1:  96.7%
+ACC: 96.7%
+MCC: 0.934
+AUC: 0.9959
+Time: 30.0 min</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB0-C2-ST
+F1:  94.6%
+ACC: 94.6%
+MCC: 0.894
+AUC: 0.9912
+Time: 29.2 min</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB0-C3-ST
+F1:  98.7%
+ACC: 98.7%
+MCC: 0.975
+AUC: 0.9989
+Time: 29.0 min</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB0-C4-ST
+F1:  95.4%
+ACC: 95.4%
+MCC: 0.908
+AUC: 0.9916
+Time: 27.7 min</t>
         </is>
       </c>
     </row>
@@ -3589,7 +3664,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB0-C4-ST
+F1:  86.1%
+ACC: 86.1%
+MCC: 0.727
+AUC: 0.8827
+Time: 19.8 min</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -3634,7 +3714,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB0-C4-ST
+F1:  95.8%
+ACC: 95.8%
+MCC: 0.917
+AUC: 0.9855
+Time: 21.8 min</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -3679,7 +3764,12 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB0-C4-ST
+F1:  95.4%
+ACC: 95.4%
+MCC: 0.908
+AUC: 0.9916
+Time: 27.7 min</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
EB0 complete on fruitvision/fruits_fresh_rotten, EB2 fruitvision started, updated trackers
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -2888,22 +2888,42 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-EB0-C1-ST
+F1:  83.6%
+ACC: 83.4%
+MCC: 0.751
+AUC: 0.9515
+Time: 68.7 min</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-EB0-C2-ST
+F1:  81.1%
+ACC: 80.7%
+MCC: 0.712
+AUC: 0.9487
+Time: 81.0 min</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-EB0-C3-ST
+F1:  91.6%
+ACC: 91.4%
+MCC: 0.872
+AUC: 0.9876
+Time: 67.4 min</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-EB0-C4-ST
+F1:  90.3%
+ACC: 90.2%
+MCC: 0.853
+AUC: 0.9822
+Time: 58.6 min</t>
         </is>
       </c>
     </row>
@@ -2958,22 +2978,42 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB0-C1-ST
+F1:  99.0%
+ACC: 99.0%
+MCC: 0.980
+AUC: 0.9996
+Time: 48.1 min</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB0-C2-ST
+F1:  98.6%
+ACC: 98.6%
+MCC: 0.973
+AUC: 0.9994
+Time: 48.5 min</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB0-C3-ST
+F1:  100.0%
+ACC: 100.0%
+MCC: 1.000
+AUC: 1.0000
+Time: 59.0 min</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB0-C4-ST
+F1:  99.7%
+ACC: 99.7%
+MCC: 0.993
+AUC: 1.0000
+Time: 48.7 min</t>
         </is>
       </c>
     </row>
@@ -3063,22 +3103,37 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB0-C1-FS
+F1:  98.5%
+ACC: 99.3%
+MCC: 0.992
+AUC: 0.9999
+Time: 81.5 min</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB0-C2-FS
+F1:  95.6%
+ACC: 97.5%
+MCC: 0.973
+AUC: 0.9995
+Time: 76.7 min</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB0-C3-FS
+F1:  98.9%
+ACC: 99.5%
+MCC: 0.995
+AUC: 0.9999
+Time: 77.8 min</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>running</t>
         </is>
       </c>
     </row>
@@ -3099,8 +3154,8 @@
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
@@ -3368,22 +3423,37 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-EB2-C1-ST
+F1:  85.5%
+ACC: 85.1%
+MCC: 0.778
+AUC: 0.9597
+Time: 80.4 min</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-EB2-C2-ST
+F1:  80.8%
+ACC: 80.4%
+MCC: 0.708
+AUC: 0.9413
+Time: 75.2 min</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-EB2-C3-ST
+F1:  92.3%
+ACC: 92.1%
+MCC: 0.881
+AUC: 0.9869
+Time: 77.8 min</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>running</t>
         </is>
       </c>
     </row>
@@ -3814,12 +3884,17 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-EB0-C4-ST
+F1:  90.3%
+ACC: 90.2%
+MCC: 0.853
+AUC: 0.9822
+Time: 58.6 min</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>running</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3934,12 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB0-C4-ST
+F1:  99.7%
+ACC: 99.7%
+MCC: 0.993
+AUC: 1.0000
+Time: 48.7 min</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update README with results summary, key findings and cross-dataset evaluation
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -3068,12 +3068,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB0-C1-ST
+F1:  97.0%
+ACC: 97.0%
+MCC: 0.941
+AUC: 0.9953
+Time: 74.4 min</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>running</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -3133,7 +3138,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>KFS-EB0-C4-FS
+F1:  95.9%
+ACC: 98.1%
+MCC: 0.980
+AUC: 0.9996
+Time: 77.6 min</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3463,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>MFV-EB2-C4-ST
+F1:  86.5%
+ACC: 86.3%
+MCC: 0.795
+AUC: 0.9685
+Time: 77.0 min</t>
         </is>
       </c>
     </row>
@@ -3508,12 +3523,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB2-C1-ST
+F1:  99.1%
+ACC: 99.2%
+MCC: 0.983
+AUC: 0.9998
+Time: 51.4 min</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>running</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -3894,7 +3914,12 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>MFV-EB2-C4-ST
+F1:  86.5%
+ACC: 86.3%
+MCC: 0.795
+AUC: 0.9685
+Time: 77.0 min</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restructure README, update LaTeX with EB0/EB2 results and new sections
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -3078,17 +3078,32 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>KFS-EB0-C2-ST
+F1:  96.3%
+ACC: 96.3%
+MCC: 0.927
+AUC: 0.9936
+Time: 78.1 min</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB0-C3-ST
+F1:  99.4%
+ACC: 99.4%
+MCC: 0.988
+AUC: 0.9997
+Time: 70.3 min</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB0-C4-ST
+F1:  98.5%
+ACC: 98.5%
+MCC: 0.970
+AUC: 0.9990
+Time: 57.4 min</t>
         </is>
       </c>
     </row>
@@ -3533,17 +3548,32 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>KFR-EB2-C2-ST
+F1:  98.6%
+ACC: 98.6%
+MCC: 0.972
+AUC: 0.9991
+Time: 55.1 min</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB2-C3-ST
+F1:  99.9%
+ACC: 99.9%
+MCC: 0.999
+AUC: 1.0000
+Time: 52.0 min</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB2-C4-ST
+F1:  99.6%
+ACC: 99.6%
+MCC: 0.991
+AUC: 1.0000
+Time: 52.1 min</t>
         </is>
       </c>
     </row>
@@ -3969,7 +3999,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-EB2-C4-ST
+F1:  99.6%
+ACC: 99.6%
+MCC: 0.991
+AUC: 1.0000
+Time: 52.1 min</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4044,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB0-C4-ST
+F1:  98.5%
+ACC: 98.5%
+MCC: 0.970
+AUC: 0.9990
+Time: 57.4 min</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update README and IEEE paper with full eval results (60 models on own_dataset)
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -3238,22 +3238,42 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB2-C1-ST
+F1:  88.9%
+ACC: 88.9%
+MCC: 0.779
+AUC: 0.9406
+Time: 18.3 min</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB2-C2-ST
+F1:  86.1%
+ACC: 86.1%
+MCC: 0.723
+AUC: 0.8897
+Time: 19.7 min</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB2-C3-ST
+F1:  88.9%
+ACC: 88.9%
+MCC: 0.789
+AUC: 0.9699
+Time: 19.8 min</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB2-C4-ST
+F1:  83.3%
+ACC: 83.3%
+MCC: 0.676
+AUC: 0.8873
+Time: 18.0 min</t>
         </is>
       </c>
     </row>
@@ -3308,22 +3328,42 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB2-C1-ST
+F1:  95.2%
+ACC: 95.2%
+MCC: 0.906
+AUC: 0.9893
+Time: 22.7 min</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB2-C2-ST
+F1:  87.0%
+ACC: 87.0%
+MCC: 0.741
+AUC: 0.9549
+Time: 23.1 min</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB2-C3-ST
+F1:  96.4%
+ACC: 96.4%
+MCC: 0.928
+AUC: 0.9947
+Time: 22.7 min</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB2-C4-ST
+F1:  92.1%
+ACC: 92.1%
+MCC: 0.843
+AUC: 0.9723
+Time: 21.1 min</t>
         </is>
       </c>
     </row>
@@ -3378,22 +3418,42 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB2-C1-ST
+F1:  96.2%
+ACC: 96.2%
+MCC: 0.924
+AUC: 0.9964
+Time: 34.4 min</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB2-C2-ST
+F1:  92.6%
+ACC: 92.6%
+MCC: 0.852
+AUC: 0.9803
+Time: 33.0 min</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB2-C3-ST
+F1:  98.0%
+ACC: 98.0%
+MCC: 0.959
+AUC: 0.9989
+Time: 34.3 min</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB2-C4-ST
+F1:  94.1%
+ACC: 94.1%
+MCC: 0.883
+AUC: 0.9882
+Time: 35.4 min</t>
         </is>
       </c>
     </row>
@@ -3628,22 +3688,42 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB2-C1-ST
+F1:  97.0%
+ACC: 97.0%
+MCC: 0.939
+AUC: 0.9962
+Time: 66.9 min</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB2-C2-ST
+F1:  96.1%
+ACC: 96.1%
+MCC: 0.921
+AUC: 0.9931
+Time: 59.1 min</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB2-C3-ST
+F1:  99.3%
+ACC: 99.3%
+MCC: 0.987
+AUC: 0.9998
+Time: 70.8 min</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB2-C4-ST
+F1:  97.9%
+ACC: 97.9%
+MCC: 0.958
+AUC: 0.9981
+Time: 62.0 min</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3874,12 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-EB2-C4-ST
+F1:  83.3%
+ACC: 83.3%
+MCC: 0.676
+AUC: 0.8873
+Time: 18.0 min</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3929,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-EB2-C4-ST
+F1:  92.1%
+ACC: 92.1%
+MCC: 0.843
+AUC: 0.9723
+Time: 21.1 min</t>
         </is>
       </c>
     </row>
@@ -3894,7 +3984,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-EB2-C4-ST
+F1:  94.1%
+ACC: 94.1%
+MCC: 0.883
+AUC: 0.9882
+Time: 35.4 min</t>
         </is>
       </c>
     </row>
@@ -4054,7 +4149,12 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-EB2-C4-ST
+F1:  97.9%
+ACC: 97.9%
+MCC: 0.958
+AUC: 0.9981
+Time: 62.0 min</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Detailed C1-C4 explanations in IEEE paper and README, analyze.py plot improvements
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -2079,8 +2079,8 @@
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
@@ -2138,22 +2138,42 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-MN3-C1-ST
+F1:  91.6%
+ACC: 91.7%
+MCC: 0.839
+AUC: 0.9591
+Time: 20.0 min</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-MN3-C2-ST
+F1:  87.4%
+ACC: 87.5%
+MCC: 0.757
+AUC: 0.9491
+Time: 19.0 min</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-MN3-C3-ST
+F1:  91.6%
+ACC: 91.7%
+MCC: 0.845
+AUC: 0.9730
+Time: 19.1 min</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-MN3-C4-ST
+F1:  86.1%
+ACC: 86.1%
+MCC: 0.741
+AUC: 0.9529
+Time: 19.0 min</t>
         </is>
       </c>
     </row>
@@ -2208,22 +2228,42 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-MN3-C1-ST
+F1:  94.6%
+ACC: 94.6%
+MCC: 0.895
+AUC: 0.9856
+Time: 22.9 min</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-MN3-C2-ST
+F1:  92.7%
+ACC: 92.7%
+MCC: 0.858
+AUC: 0.9774
+Time: 23.1 min</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-MN3-C3-ST
+F1:  96.7%
+ACC: 96.7%
+MCC: 0.934
+AUC: 0.9969
+Time: 27.0 min</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-MN3-C4-ST
+F1:  95.8%
+ACC: 95.8%
+MCC: 0.917
+AUC: 0.9852
+Time: 24.6 min</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2318,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-MN3-C1-ST
+F1:  94.4%
+ACC: 94.4%
+MCC: 0.892
+AUC: 0.9936
+Time: 33.9 min</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2348,22 +2393,42 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-MN3-C1-ST
+F1:  83.3%
+ACC: 82.9%
+MCC: 0.746
+AUC: 0.9549
+Time: 60.5 min</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-MN3-C2-ST
+F1:  80.9%
+ACC: 80.5%
+MCC: 0.711
+AUC: 0.9460
+Time: 59.0 min</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-MN3-C3-ST
+F1:  92.4%
+ACC: 92.3%
+MCC: 0.884
+AUC: 0.9893
+Time: 67.8 min</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-MN3-C4-ST
+F1:  89.4%
+ACC: 89.3%
+MCC: 0.840
+AUC: 0.9768
+Time: 66.5 min</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3924,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFQ-MN3-C4-ST
+F1:  86.1%
+ACC: 86.1%
+MCC: 0.741
+AUC: 0.9529
+Time: 19.0 min</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -3914,7 +3984,12 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFR-MN3-C4-ST
+F1:  95.8%
+ACC: 95.8%
+MCC: 0.917
+AUC: 0.9852
+Time: 24.6 min</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -4024,7 +4099,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MFV-MN3-C4-ST
+F1:  89.4%
+ACC: 89.3%
+MCC: 0.840
+AUC: 0.9768
+Time: 66.5 min</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add glossary.tex/pdf with acronyms and key concepts
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -2328,17 +2328,32 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-MN3-C2-ST
+F1:  91.0%
+ACC: 91.0%
+MCC: 0.828
+AUC: 0.9722
+Time: 44.5 min</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-MN3-C3-ST
+F1:  98.2%
+ACC: 98.2%
+MCC: 0.964
+AUC: 0.9984
+Time: 34.2 min</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-MN3-C4-ST
+F1:  92.8%
+ACC: 92.8%
+MCC: 0.863
+AUC: 0.9866
+Time: 36.1 min</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2498,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>running</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -2553,12 +2568,22 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-MN3-C1-ST
+F1:  95.9%
+ACC: 96.0%
+MCC: 0.919
+AUC: 0.9928
+Time: 75.0 min</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-MN3-C2-ST
+F1:  93.4%
+ACC: 93.5%
+MCC: 0.869
+AUC: 0.9828
+Time: 67.4 min</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4044,7 +4069,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>MLM-MN3-C4-ST
+F1:  92.8%
+ACC: 92.8%
+MCC: 0.863
+AUC: 0.9866
+Time: 36.1 min</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add confidence distribution explanation and R34/R50 notes to Excel legends
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -2498,12 +2498,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>KFR-MN3-C1-ST
+F1:  99.1%
+ACC: 99.1%
+MCC: 0.982
+AUC: 0.9995
+Time: 47.5 min</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>running</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4279,7 +4284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -4769,10 +4774,91 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>BACKBONE NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>R18 (ResNet-18)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Primary baseline. 11.2M params, 512-dim output. All experiments complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>EB0 (EfficientNet-B0)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Phase 2 backbone. 5.3M params, 1280-dim output. All experiments complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>EB2 (EfficientNet-B2)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Phase 2 backbone. 9.1M params, 1408-dim output. All experiments complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>MN3 (MobileNetV3-S)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Lightweight backbone for edge/mobile deployment. 2.5M params, 576-dim output. Experiments in progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>R34 (ResNet-34)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>NOT CURRENTLY EVALUATED. Included in registry for future use. Similar architecture to R18 with more layers (21.3M params). Expected to perform marginally better than R18 but at higher computational cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>R50 (ResNet-50)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>NOT CURRENTLY EVALUATED. Included in registry for future use. Deeper ResNet variant (25.6M params, 2048-dim output). Uses bottleneck blocks; better suited for large datasets.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A52:B52"/>
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A37:B37"/>

</xml_diff>

<commit_message>
Remove ResNet-34 and ResNet-50 from all files. Add --eval flag to analyze.py.
</commit_message>
<xml_diff>
--- a/experiments_tracker.xlsx
+++ b/experiments_tracker.xlsx
@@ -2508,17 +2508,32 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>KFR-MN3-C2-ST
+F1:  97.8%
+ACC: 97.9%
+MCC: 0.957
+AUC: 0.9973
+Time: 45.5 min</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-MN3-C3-ST
+F1:  100.0%
+ACC: 100.0%
+MCC: 1.000
+AUC: 1.0000
+Time: 53.0 min</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-MN3-C4-ST
+F1:  99.4%
+ACC: 99.4%
+MCC: 0.989
+AUC: 0.9998
+Time: 56.0 min</t>
         </is>
       </c>
     </row>
@@ -2593,12 +2608,22 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-MN3-C3-ST
+F1:  99.2%
+ACC: 99.2%
+MCC: 0.984
+AUC: 0.9996
+Time: 75.0 min</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-MN3-C4-ST
+F1:  97.8%
+ACC: 97.8%
+MCC: 0.955
+AUC: 0.9983
+Time: 69.7 min</t>
         </is>
       </c>
     </row>
@@ -4194,7 +4219,12 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFR-MN3-C4-ST
+F1:  99.4%
+ACC: 99.4%
+MCC: 0.989
+AUC: 0.9998
+Time: 56.0 min</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -4249,7 +4279,12 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>KFS-MN3-C4-ST
+F1:  97.8%
+ACC: 97.8%
+MCC: 0.955
+AUC: 0.9983
+Time: 69.7 min</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">

</xml_diff>